<commit_message>
Updated cases and excel file
</commit_message>
<xml_diff>
--- a/DebeersUSUAT/US - Test Case Summary.xlsx
+++ b/DebeersUSUAT/US - Test Case Summary.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlayWright Python\DebeersUSUAT\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8191AF53-54FD-4B98-AFBB-1486E22187FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Menu and Header" sheetId="1" r:id="rId1"/>
+    <sheet name="Checkout as Guest" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +25,134 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+  <si>
+    <t>Case #</t>
+  </si>
+  <si>
+    <t>Case Summary</t>
+  </si>
+  <si>
+    <t>Open URL. Accept Cookie Consent. Close Country Selector and Email Subscription popups.</t>
+  </si>
+  <si>
+    <t>From the Menu &gt; Open and Close Store Locator page.</t>
+  </si>
+  <si>
+    <t>From the Menu &gt; Open Book an Appointment page.</t>
+  </si>
+  <si>
+    <t>Select all book an appointment options with In Store appointment type. Open and Close Map marker.</t>
+  </si>
+  <si>
+    <t>Select all book an appointment options with Virtual appointment type. Open and Close Map marker.</t>
+  </si>
+  <si>
+    <t>From the Menu &gt; Open Delivery and Returns page.</t>
+  </si>
+  <si>
+    <t>From the Menu &gt; Open Contact Us page. Change regions.</t>
+  </si>
+  <si>
+    <t>From the Menu &gt; Change Languages.</t>
+  </si>
+  <si>
+    <t>From the Menu &gt; Change Locations.</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Amex card + Same Billing address</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Visa card + Use Delivery address as Billing address</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Union Pay card + Different Billing address.</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Discover card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Master card &gt; From the Payment page, Go back to the Delivery Page &gt; Premium Delivery + Discover card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Master card &gt; From the Payment page, Go back to the Delivery Page &gt; Change delivery method to Self Collect + Discover card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Master card &gt; From the Payment page, Go back to the Delivery Page &gt; Change delivery method to Someone Else Collect + Discover card</t>
+  </si>
+  <si>
+    <t>Self Collect + Union Pay card &gt; From the Payment page, Go back to the Delivery Page &gt; Self Collect + Amex card</t>
+  </si>
+  <si>
+    <t>Self Collect + Union Pay card &gt; From the Payment page, Go back to the Delivery Page &gt; Change delivery method to Premium Delivery + Amex card</t>
+  </si>
+  <si>
+    <t>Self Collect + Union Pay card &gt; From the Payment page, Go back to the Delivery Page &gt; Change delivery method to Someone Else Collect + Amex card</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Visa card &gt; From the Payment page, Go back to the Delivery Page &gt; Someone Else Collect + Union Pay card</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Visa card &gt; From the Payment page, Go back to the Delivery Page &gt; Change delivery method to Premium Delivery + Union Pay card</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Visa card &gt; From the Payment page, Go back to the Delivery Page &gt; Change delivery method to Self Collect + Union Pay card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Discover card &gt; From the Review page, Go back to the Delivery Page &gt; Premium Delivery + Master card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Discover card &gt; From the Review page, Go back to the Delivery Page &gt; Change delivery method to Self Collect + Master card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Discover card &gt; From the Review page, Go back to the Delivery Page &gt; Change delivery method to Someone Else Collect + Master card</t>
+  </si>
+  <si>
+    <t>Self Collect + Amex card &gt; From the Review page, Go back to the Delivery Page &gt; Self Collect + Union Pay card</t>
+  </si>
+  <si>
+    <t>Self Collect + Amex card &gt; From the Review page, Go back to the Delivery Page &gt; Change delivery method to Premium Delivery + Union Pay card</t>
+  </si>
+  <si>
+    <t>Self Collect + Amex card &gt; From the Review page, Go back to the Delivery Page &gt; Change delivery method to Someone Else Collect + Union Pay card</t>
+  </si>
+  <si>
+    <t>Self Collect + Master card + Same Billing Name</t>
+  </si>
+  <si>
+    <t>Self Collect + Master card + Different Billing Name</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Union Pay card &gt; From the Review page, Go back to the Delivery Page &gt; Someone Else Collect + Visa card</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Union Pay card &gt; From the Review page, Go back to the Delivery Page &gt; Change delivery method to Premium Delivery + Visa card</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Union Pay card &gt; From the Review page, Go back to the Delivery Page &gt; Change delivery method to Self Collect + Visa card</t>
+  </si>
+  <si>
+    <t>Someone Else Collect + Discover card &gt; From the Review page, Go back to the Payment Page &gt; Visa card</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Master card &gt; From the Review page, Go back to the Payment Page &gt; Discover card + Use Delivery address as Billing address</t>
+  </si>
+  <si>
+    <t>Premium Delivery + Discover card &gt; From the Review page, Go back to the Payment Page &gt; Master card + Different name and address</t>
+  </si>
+  <si>
+    <t>Self Collect + Union Pay card &gt; From the Review page, Go back to the Payment Page &gt; Amex card + Same Billing name</t>
+  </si>
+  <si>
+    <t>Self Collect + Amex card &gt; From the Review page, Go back to the Payment Page &gt; Union Pay card + Different Billing name</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +160,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +191,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +512,400 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="6.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.28515625" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64825CBC-1DCE-405C-BBF9-8B8B7348A5D2}">
+  <dimension ref="A1:B38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="3"/>
+    <col min="2" max="2" width="183.140625" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="5"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" s="5"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="5"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35" s="5"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>35</v>
+      </c>
+      <c r="B36" s="5"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>36</v>
+      </c>
+      <c r="B37" s="5"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>